<commit_message>
feat: refresh report layout and sales window metrics
</commit_message>
<xml_diff>
--- a/data/sku装箱数.xlsx
+++ b/data/sku装箱数.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11109"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\62625\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/armewang/Documents/CS-Tech/Local/pseudoctor-sale-inventory-reviewer/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95A38DE7-A5CA-4EF2-8169-17503B3B98FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0323F50F-0DAF-5043-ACE8-4578A3617396}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="19396" windowHeight="11475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="78">
   <si>
     <t>品牌</t>
   </si>
@@ -262,6 +262,12 @@
   <si>
     <t>秦俑275g袋装中老年粉275g</t>
     <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>6907992642291</t>
+  </si>
+  <si>
+    <t>伊利纯牛奶粉700g</t>
   </si>
 </sst>
 </file>
@@ -272,14 +278,14 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="14"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="4"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -288,27 +294,33 @@
       <b/>
       <sz val="14"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -368,13 +380,28 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -396,9 +423,21 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -671,17 +710,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D35"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="17.649999999999999" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:D36"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="19" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11" style="1" customWidth="1"/>
-    <col min="2" max="2" width="26.46875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="38.64453125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.8203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="26.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="38.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.83203125" style="1" customWidth="1"/>
     <col min="5" max="16384" width="11" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -695,7 +734,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
@@ -709,7 +748,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="5"/>
       <c r="B3" s="2" t="s">
         <v>6</v>
@@ -721,7 +760,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="5"/>
       <c r="B4" s="2" t="s">
         <v>8</v>
@@ -733,7 +772,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="5"/>
       <c r="B5" s="2" t="s">
         <v>10</v>
@@ -745,7 +784,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" s="5"/>
       <c r="B6" s="2" t="s">
         <v>12</v>
@@ -757,7 +796,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" s="5"/>
       <c r="B7" s="2" t="s">
         <v>14</v>
@@ -769,7 +808,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" s="5"/>
       <c r="B8" s="2" t="s">
         <v>16</v>
@@ -781,7 +820,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" s="5"/>
       <c r="B9" s="2" t="s">
         <v>18</v>
@@ -793,7 +832,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" s="5"/>
       <c r="B10" s="2" t="s">
         <v>20</v>
@@ -805,7 +844,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" s="5"/>
       <c r="B11" s="2" t="s">
         <v>22</v>
@@ -817,7 +856,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" s="5"/>
       <c r="B12" s="2" t="s">
         <v>24</v>
@@ -829,7 +868,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" s="5"/>
       <c r="B13" s="2" t="s">
         <v>26</v>
@@ -841,7 +880,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" s="5"/>
       <c r="B14" s="2" t="s">
         <v>28</v>
@@ -853,7 +892,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" s="5"/>
       <c r="B15" s="2" t="s">
         <v>30</v>
@@ -865,7 +904,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" s="5"/>
       <c r="B16" s="2" t="s">
         <v>32</v>
@@ -877,7 +916,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" s="5"/>
       <c r="B17" s="2" t="s">
         <v>34</v>
@@ -889,7 +928,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="5"/>
       <c r="B18" s="2" t="s">
         <v>36</v>
@@ -901,7 +940,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" s="5"/>
       <c r="B19" s="2" t="s">
         <v>38</v>
@@ -913,7 +952,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" s="5"/>
       <c r="B20" s="2" t="s">
         <v>40</v>
@@ -925,7 +964,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" s="6"/>
       <c r="B21" s="2" t="s">
         <v>42</v>
@@ -937,185 +976,197 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A22" s="2" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D22" s="10"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B23" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C23" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D22" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A23" s="4" t="s">
+      <c r="D23" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C24" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D23" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A24" s="5"/>
-      <c r="B24" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>51</v>
-      </c>
       <c r="D24" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" s="5"/>
       <c r="B25" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D25" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" s="5"/>
       <c r="B26" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D26" s="2">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" s="5"/>
       <c r="B27" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D27" s="2">
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" s="5"/>
       <c r="B28" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D28" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" s="5"/>
       <c r="B29" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D29" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" s="5"/>
       <c r="B30" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D30" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A31" s="5"/>
+      <c r="B31" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C31" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D30" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A31" s="6"/>
-      <c r="B31" s="2" t="s">
+      <c r="D31" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A32" s="6"/>
+      <c r="B32" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="C31" s="2" t="s">
+      <c r="C32" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="D31" s="2">
+      <c r="D32" s="2">
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A32" s="4" t="s">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B33" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C33" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D32" s="2">
+      <c r="D33" s="2">
         <v>24</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A33" s="5"/>
-      <c r="B33" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D33" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A34" s="5"/>
       <c r="B34" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D34" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A35" s="5"/>
+      <c r="B35" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="D34" s="2">
+      <c r="D35" s="2">
         <v>24</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.4">
-      <c r="A35" s="6"/>
-      <c r="B35" s="2" t="s">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A36" s="6"/>
+      <c r="B36" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="C35" s="2" t="s">
+      <c r="C36" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D36" s="2">
         <v>24</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A2:A21"/>
-    <mergeCell ref="A23:A31"/>
-    <mergeCell ref="A32:A35"/>
+    <mergeCell ref="A24:A32"/>
+    <mergeCell ref="A33:A36"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>